<commit_message>
ejecucion para el dia lunes 15 de agosto del 2026 agrergando la consulta para creacion de tablas en BI para su consulta por parte del equipo con todos los campos del portal detecno
</commit_message>
<xml_diff>
--- a/detecno.xlsx
+++ b/detecno.xlsx
@@ -5,13 +5,13 @@
     <workbookView/>
   </bookViews>
   <sheets>
-    <sheet name="Facturas Seleccionadas" sheetId="1" r:id="R1f2356bc337d4019"/>
+    <sheet name="Facturas Seleccionadas" sheetId="1" r:id="R713e6318263c4ab1"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1950" uniqueCount="1950">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2034" uniqueCount="2034">
   <si>
     <t>ID</t>
   </si>
@@ -5861,6 +5861,258 @@
   </si>
   <si>
     <t>4500472948</t>
+  </si>
+  <si>
+    <t>49441</t>
+  </si>
+  <si>
+    <t>2d125b66-daaf-4250-a894-6bac818fee23</t>
+  </si>
+  <si>
+    <t>E006325064</t>
+  </si>
+  <si>
+    <t>49452</t>
+  </si>
+  <si>
+    <t>2ded3c00-0adc-47d0-875a-ea429509c4d8</t>
+  </si>
+  <si>
+    <t>10092291</t>
+  </si>
+  <si>
+    <t>49658</t>
+  </si>
+  <si>
+    <t>2a5d7bc0-7834-4ac0-8070-812ca89e1e42</t>
+  </si>
+  <si>
+    <t>E006332709</t>
+  </si>
+  <si>
+    <t>49656</t>
+  </si>
+  <si>
+    <t>2346aba1-483a-4dcf-9557-d284bfc3ca48</t>
+  </si>
+  <si>
+    <t>E006332710</t>
+  </si>
+  <si>
+    <t>49824</t>
+  </si>
+  <si>
+    <t>6fe2ae18-3d72-48ee-bd35-47354c3a90a2</t>
+  </si>
+  <si>
+    <t>E006332700</t>
+  </si>
+  <si>
+    <t>49822</t>
+  </si>
+  <si>
+    <t>336bd384-f59e-4f82-a2d8-6f6cf3dd1338</t>
+  </si>
+  <si>
+    <t>E006332715</t>
+  </si>
+  <si>
+    <t>49798</t>
+  </si>
+  <si>
+    <t>3289abf6-c4c2-4fa0-9282-8e2a8e3b1be1</t>
+  </si>
+  <si>
+    <t>E006332702</t>
+  </si>
+  <si>
+    <t>49773</t>
+  </si>
+  <si>
+    <t>d84badf0-9272-4c19-879a-3a2289ac9df0</t>
+  </si>
+  <si>
+    <t>E006332704</t>
+  </si>
+  <si>
+    <t>49772</t>
+  </si>
+  <si>
+    <t>ca9ad7d9-867a-4d44-992c-de3430024c26</t>
+  </si>
+  <si>
+    <t>E006332706</t>
+  </si>
+  <si>
+    <t>49795</t>
+  </si>
+  <si>
+    <t>011a4ce3-ca2c-48b2-9200-e8b4bb23a809</t>
+  </si>
+  <si>
+    <t>E006332703</t>
+  </si>
+  <si>
+    <t>49771</t>
+  </si>
+  <si>
+    <t>27653a3b-a13c-4dcc-ab81-896182873606</t>
+  </si>
+  <si>
+    <t>E006332708</t>
+  </si>
+  <si>
+    <t>49793</t>
+  </si>
+  <si>
+    <t>bbde6942-2c76-402e-af97-af7117044bf3</t>
+  </si>
+  <si>
+    <t>E006332705</t>
+  </si>
+  <si>
+    <t>49181</t>
+  </si>
+  <si>
+    <t>5bf772dd-f8d9-403a-aada-83b86aade1bc</t>
+  </si>
+  <si>
+    <t>E006332714</t>
+  </si>
+  <si>
+    <t>49636</t>
+  </si>
+  <si>
+    <t>02ca9f13-e60c-49a4-9dc1-558ebb2d7e88</t>
+  </si>
+  <si>
+    <t>E006332711</t>
+  </si>
+  <si>
+    <t>49770</t>
+  </si>
+  <si>
+    <t>f6790e1d-4653-4743-98e3-7774b9d031ee</t>
+  </si>
+  <si>
+    <t>E006332707</t>
+  </si>
+  <si>
+    <t>49821</t>
+  </si>
+  <si>
+    <t>37b26d13-ab25-4516-ab03-9db548e69567</t>
+  </si>
+  <si>
+    <t>E006332719</t>
+  </si>
+  <si>
+    <t>49831</t>
+  </si>
+  <si>
+    <t>dd8148f5-1a57-4f09-bfe1-2e0599e2f7b8</t>
+  </si>
+  <si>
+    <t>E006332716</t>
+  </si>
+  <si>
+    <t>49896</t>
+  </si>
+  <si>
+    <t>7d242e74-0941-4215-a22c-7f5878dcfe44</t>
+  </si>
+  <si>
+    <t>E006332701</t>
+  </si>
+  <si>
+    <t>50125</t>
+  </si>
+  <si>
+    <t>f493a15f-8ab2-408c-a335-b70095c1ddf7</t>
+  </si>
+  <si>
+    <t>4500483949</t>
+  </si>
+  <si>
+    <t>49999</t>
+  </si>
+  <si>
+    <t>719fc77b-ddc6-4c68-859e-09905305b398</t>
+  </si>
+  <si>
+    <t>4500462983</t>
+  </si>
+  <si>
+    <t>49551</t>
+  </si>
+  <si>
+    <t>e15cf424-cb33-4856-804f-a5b1093a7d31</t>
+  </si>
+  <si>
+    <t>E006326885</t>
+  </si>
+  <si>
+    <t>49512</t>
+  </si>
+  <si>
+    <t>b94d18cf-9570-4ee0-be47-09ea324f9c52</t>
+  </si>
+  <si>
+    <t>E006332713</t>
+  </si>
+  <si>
+    <t>49995</t>
+  </si>
+  <si>
+    <t>29fff213-3f86-41bf-83c0-528cf03937e4</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>50035</t>
+  </si>
+  <si>
+    <t>bd4eeb32-33f3-43a3-8f6b-2a71638b7534</t>
+  </si>
+  <si>
+    <t>4500458230</t>
+  </si>
+  <si>
+    <t>50053</t>
+  </si>
+  <si>
+    <t>28ba7ec4-1ce1-4578-aa63-b7d8587d5f65</t>
+  </si>
+  <si>
+    <t>4500480141</t>
+  </si>
+  <si>
+    <t>50122</t>
+  </si>
+  <si>
+    <t>700d11a0-d9ec-48c1-8213-b0becadd3e8b</t>
+  </si>
+  <si>
+    <t>4500480562</t>
+  </si>
+  <si>
+    <t>50118</t>
+  </si>
+  <si>
+    <t>dcacc4a3-64b5-4dfe-b99d-c82dd2e05a0a</t>
+  </si>
+  <si>
+    <t>4500480569</t>
+  </si>
+  <si>
+    <t>50222</t>
+  </si>
+  <si>
+    <t>a1e34d93-b3ca-4908-9f96-1914ae77ca7e</t>
+  </si>
+  <si>
+    <t>4500460559</t>
   </si>
 </sst>
 </file>
@@ -5906,7 +6158,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AG674"/>
+  <dimension ref="A1:AG702"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.140625" customWidth="1"/>
@@ -74018,6 +74270,2834 @@
         <v>43</v>
       </c>
     </row>
+    <row r="675">
+      <c r="A675" s="0">
+        <v>18697</v>
+      </c>
+      <c r="B675" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C675" s="0" t="s">
+        <v>1950</v>
+      </c>
+      <c r="D675" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E675" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F675" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G675" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H675" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I675" s="0">
+        <v>20260814</v>
+      </c>
+      <c r="J675" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="K675" s="0">
+        <v>70977.56</v>
+      </c>
+      <c r="L675" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M675" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N675" s="0" t="s">
+        <v>1951</v>
+      </c>
+      <c r="O675" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P675" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q675" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R675" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S675" s="0">
+        <v>20260814</v>
+      </c>
+      <c r="T675" s="0">
+        <v>9790.01</v>
+      </c>
+      <c r="U675" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V675" s="0">
+        <v>1</v>
+      </c>
+      <c r="W675" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X675" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y675" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z675" s="0">
+        <v>70977.56</v>
+      </c>
+      <c r="AA675" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB675" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC675" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD675" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="AE675" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF675" s="0" t="s">
+        <v>1952</v>
+      </c>
+      <c r="AG675" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" s="0">
+        <v>19114</v>
+      </c>
+      <c r="B676" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C676" s="0" t="s">
+        <v>1953</v>
+      </c>
+      <c r="D676" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E676" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F676" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G676" s="0" t="s">
+        <v>560</v>
+      </c>
+      <c r="H676" s="0" t="s">
+        <v>561</v>
+      </c>
+      <c r="I676" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J676" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K676" s="0">
+        <v>40931.45</v>
+      </c>
+      <c r="L676" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M676" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N676" s="0" t="s">
+        <v>1954</v>
+      </c>
+      <c r="O676" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P676" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q676" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R676" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S676" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T676" s="0">
+        <v>5645.71</v>
+      </c>
+      <c r="U676" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V676" s="0">
+        <v>1</v>
+      </c>
+      <c r="W676" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X676" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y676" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z676" s="0">
+        <v>40931.45</v>
+      </c>
+      <c r="AA676" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB676" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC676" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD676" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE676" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF676" s="0" t="s">
+        <v>1955</v>
+      </c>
+      <c r="AG676" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" s="0">
+        <v>19115</v>
+      </c>
+      <c r="B677" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C677" s="0" t="s">
+        <v>1956</v>
+      </c>
+      <c r="D677" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E677" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F677" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G677" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H677" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I677" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J677" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K677" s="0">
+        <v>13670.27</v>
+      </c>
+      <c r="L677" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M677" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N677" s="0" t="s">
+        <v>1957</v>
+      </c>
+      <c r="O677" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P677" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q677" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R677" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S677" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T677" s="0">
+        <v>1885.56</v>
+      </c>
+      <c r="U677" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V677" s="0">
+        <v>1</v>
+      </c>
+      <c r="W677" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X677" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y677" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z677" s="0">
+        <v>13670.27</v>
+      </c>
+      <c r="AA677" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB677" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC677" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD677" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE677" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF677" s="0" t="s">
+        <v>1958</v>
+      </c>
+      <c r="AG677" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="0">
+        <v>19116</v>
+      </c>
+      <c r="B678" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C678" s="0" t="s">
+        <v>1959</v>
+      </c>
+      <c r="D678" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E678" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F678" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G678" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H678" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I678" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J678" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K678" s="0">
+        <v>12858.27</v>
+      </c>
+      <c r="L678" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M678" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N678" s="0" t="s">
+        <v>1960</v>
+      </c>
+      <c r="O678" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P678" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q678" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R678" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S678" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T678" s="0">
+        <v>1773.56</v>
+      </c>
+      <c r="U678" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V678" s="0">
+        <v>1</v>
+      </c>
+      <c r="W678" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X678" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y678" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z678" s="0">
+        <v>12858.27</v>
+      </c>
+      <c r="AA678" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB678" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC678" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD678" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE678" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF678" s="0" t="s">
+        <v>1961</v>
+      </c>
+      <c r="AG678" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="0">
+        <v>19117</v>
+      </c>
+      <c r="B679" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C679" s="0" t="s">
+        <v>1962</v>
+      </c>
+      <c r="D679" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E679" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F679" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G679" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H679" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I679" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J679" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K679" s="0">
+        <v>12858.27</v>
+      </c>
+      <c r="L679" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M679" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N679" s="0" t="s">
+        <v>1963</v>
+      </c>
+      <c r="O679" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P679" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q679" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R679" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S679" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T679" s="0">
+        <v>1773.56</v>
+      </c>
+      <c r="U679" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V679" s="0">
+        <v>1</v>
+      </c>
+      <c r="W679" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X679" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y679" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z679" s="0">
+        <v>12858.27</v>
+      </c>
+      <c r="AA679" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB679" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC679" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD679" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE679" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF679" s="0" t="s">
+        <v>1964</v>
+      </c>
+      <c r="AG679" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="0">
+        <v>19118</v>
+      </c>
+      <c r="B680" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C680" s="0" t="s">
+        <v>1965</v>
+      </c>
+      <c r="D680" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E680" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F680" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G680" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H680" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I680" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J680" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K680" s="0">
+        <v>12858.27</v>
+      </c>
+      <c r="L680" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M680" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N680" s="0" t="s">
+        <v>1966</v>
+      </c>
+      <c r="O680" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P680" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q680" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R680" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S680" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T680" s="0">
+        <v>1773.56</v>
+      </c>
+      <c r="U680" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V680" s="0">
+        <v>1</v>
+      </c>
+      <c r="W680" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X680" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y680" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z680" s="0">
+        <v>12858.27</v>
+      </c>
+      <c r="AA680" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB680" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC680" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD680" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE680" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF680" s="0" t="s">
+        <v>1967</v>
+      </c>
+      <c r="AG680" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="0">
+        <v>19119</v>
+      </c>
+      <c r="B681" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C681" s="0" t="s">
+        <v>1968</v>
+      </c>
+      <c r="D681" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E681" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F681" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G681" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H681" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I681" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J681" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K681" s="0">
+        <v>21039.7</v>
+      </c>
+      <c r="L681" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M681" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N681" s="0" t="s">
+        <v>1969</v>
+      </c>
+      <c r="O681" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P681" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q681" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R681" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S681" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T681" s="0">
+        <v>2902.03</v>
+      </c>
+      <c r="U681" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V681" s="0">
+        <v>1</v>
+      </c>
+      <c r="W681" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X681" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y681" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z681" s="0">
+        <v>21039.7</v>
+      </c>
+      <c r="AA681" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB681" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC681" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD681" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE681" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF681" s="0" t="s">
+        <v>1970</v>
+      </c>
+      <c r="AG681" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" s="0">
+        <v>19120</v>
+      </c>
+      <c r="B682" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C682" s="0" t="s">
+        <v>1971</v>
+      </c>
+      <c r="D682" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E682" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F682" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G682" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H682" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I682" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J682" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K682" s="0">
+        <v>20685.9</v>
+      </c>
+      <c r="L682" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M682" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N682" s="0" t="s">
+        <v>1972</v>
+      </c>
+      <c r="O682" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P682" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q682" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R682" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S682" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T682" s="0">
+        <v>2853.23</v>
+      </c>
+      <c r="U682" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V682" s="0">
+        <v>1</v>
+      </c>
+      <c r="W682" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X682" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y682" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z682" s="0">
+        <v>20685.9</v>
+      </c>
+      <c r="AA682" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB682" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC682" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD682" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE682" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF682" s="0" t="s">
+        <v>1973</v>
+      </c>
+      <c r="AG682" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" s="0">
+        <v>19121</v>
+      </c>
+      <c r="B683" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C683" s="0" t="s">
+        <v>1974</v>
+      </c>
+      <c r="D683" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E683" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F683" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G683" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H683" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I683" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J683" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K683" s="0">
+        <v>20685.9</v>
+      </c>
+      <c r="L683" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M683" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N683" s="0" t="s">
+        <v>1975</v>
+      </c>
+      <c r="O683" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P683" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q683" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R683" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S683" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T683" s="0">
+        <v>2853.23</v>
+      </c>
+      <c r="U683" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V683" s="0">
+        <v>1</v>
+      </c>
+      <c r="W683" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X683" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y683" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z683" s="0">
+        <v>20685.9</v>
+      </c>
+      <c r="AA683" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB683" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC683" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD683" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE683" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF683" s="0" t="s">
+        <v>1976</v>
+      </c>
+      <c r="AG683" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" s="0">
+        <v>19122</v>
+      </c>
+      <c r="B684" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C684" s="0" t="s">
+        <v>1977</v>
+      </c>
+      <c r="D684" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E684" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F684" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G684" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H684" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I684" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J684" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K684" s="0">
+        <v>12950.16</v>
+      </c>
+      <c r="L684" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M684" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N684" s="0" t="s">
+        <v>1978</v>
+      </c>
+      <c r="O684" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P684" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q684" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R684" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S684" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T684" s="0">
+        <v>1786.23</v>
+      </c>
+      <c r="U684" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V684" s="0">
+        <v>1</v>
+      </c>
+      <c r="W684" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X684" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y684" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z684" s="0">
+        <v>12950.16</v>
+      </c>
+      <c r="AA684" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB684" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC684" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD684" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE684" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF684" s="0" t="s">
+        <v>1979</v>
+      </c>
+      <c r="AG684" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="0">
+        <v>19123</v>
+      </c>
+      <c r="B685" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C685" s="0" t="s">
+        <v>1980</v>
+      </c>
+      <c r="D685" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E685" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F685" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G685" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H685" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I685" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J685" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K685" s="0">
+        <v>20685.9</v>
+      </c>
+      <c r="L685" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M685" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N685" s="0" t="s">
+        <v>1981</v>
+      </c>
+      <c r="O685" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P685" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q685" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R685" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S685" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T685" s="0">
+        <v>2853.23</v>
+      </c>
+      <c r="U685" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V685" s="0">
+        <v>1</v>
+      </c>
+      <c r="W685" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X685" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y685" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z685" s="0">
+        <v>20685.9</v>
+      </c>
+      <c r="AA685" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB685" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC685" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD685" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE685" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF685" s="0" t="s">
+        <v>1982</v>
+      </c>
+      <c r="AG685" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" s="0">
+        <v>19125</v>
+      </c>
+      <c r="B686" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C686" s="0" t="s">
+        <v>1983</v>
+      </c>
+      <c r="D686" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E686" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F686" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G686" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H686" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I686" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J686" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K686" s="0">
+        <v>20685.9</v>
+      </c>
+      <c r="L686" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M686" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N686" s="0" t="s">
+        <v>1984</v>
+      </c>
+      <c r="O686" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P686" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q686" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R686" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S686" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T686" s="0">
+        <v>2853.23</v>
+      </c>
+      <c r="U686" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V686" s="0">
+        <v>1</v>
+      </c>
+      <c r="W686" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X686" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y686" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z686" s="0">
+        <v>20685.9</v>
+      </c>
+      <c r="AA686" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB686" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC686" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD686" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE686" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF686" s="0" t="s">
+        <v>1985</v>
+      </c>
+      <c r="AG686" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" s="0">
+        <v>19126</v>
+      </c>
+      <c r="B687" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C687" s="0" t="s">
+        <v>1986</v>
+      </c>
+      <c r="D687" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E687" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F687" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G687" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H687" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I687" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J687" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K687" s="0">
+        <v>21911.88</v>
+      </c>
+      <c r="L687" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M687" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N687" s="0" t="s">
+        <v>1987</v>
+      </c>
+      <c r="O687" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P687" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q687" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R687" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S687" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T687" s="0">
+        <v>3022.33</v>
+      </c>
+      <c r="U687" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V687" s="0">
+        <v>1</v>
+      </c>
+      <c r="W687" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X687" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y687" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z687" s="0">
+        <v>21911.88</v>
+      </c>
+      <c r="AA687" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB687" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC687" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD687" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE687" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF687" s="0" t="s">
+        <v>1988</v>
+      </c>
+      <c r="AG687" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="0">
+        <v>19127</v>
+      </c>
+      <c r="B688" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C688" s="0" t="s">
+        <v>1989</v>
+      </c>
+      <c r="D688" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E688" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F688" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G688" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H688" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I688" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J688" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K688" s="0">
+        <v>18923.82</v>
+      </c>
+      <c r="L688" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M688" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N688" s="0" t="s">
+        <v>1990</v>
+      </c>
+      <c r="O688" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P688" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q688" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R688" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S688" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T688" s="0">
+        <v>2610.18</v>
+      </c>
+      <c r="U688" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V688" s="0">
+        <v>1</v>
+      </c>
+      <c r="W688" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X688" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y688" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z688" s="0">
+        <v>18923.82</v>
+      </c>
+      <c r="AA688" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB688" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC688" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD688" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE688" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF688" s="0" t="s">
+        <v>1991</v>
+      </c>
+      <c r="AG688" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="0">
+        <v>19128</v>
+      </c>
+      <c r="B689" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C689" s="0" t="s">
+        <v>1992</v>
+      </c>
+      <c r="D689" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E689" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F689" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G689" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H689" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I689" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J689" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K689" s="0">
+        <v>9918.7</v>
+      </c>
+      <c r="L689" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M689" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N689" s="0" t="s">
+        <v>1993</v>
+      </c>
+      <c r="O689" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P689" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q689" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R689" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S689" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T689" s="0">
+        <v>1368.1</v>
+      </c>
+      <c r="U689" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V689" s="0">
+        <v>1</v>
+      </c>
+      <c r="W689" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X689" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y689" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z689" s="0">
+        <v>9918.7</v>
+      </c>
+      <c r="AA689" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB689" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC689" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD689" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE689" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF689" s="0" t="s">
+        <v>1994</v>
+      </c>
+      <c r="AG689" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="0">
+        <v>19130</v>
+      </c>
+      <c r="B690" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C690" s="0" t="s">
+        <v>1995</v>
+      </c>
+      <c r="D690" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E690" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F690" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G690" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H690" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I690" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J690" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K690" s="0">
+        <v>19072.25</v>
+      </c>
+      <c r="L690" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M690" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N690" s="0" t="s">
+        <v>1996</v>
+      </c>
+      <c r="O690" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P690" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q690" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R690" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S690" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T690" s="0">
+        <v>2630.66</v>
+      </c>
+      <c r="U690" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V690" s="0">
+        <v>1</v>
+      </c>
+      <c r="W690" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X690" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y690" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z690" s="0">
+        <v>19072.25</v>
+      </c>
+      <c r="AA690" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB690" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC690" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD690" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE690" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF690" s="0" t="s">
+        <v>1997</v>
+      </c>
+      <c r="AG690" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" s="0">
+        <v>19131</v>
+      </c>
+      <c r="B691" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C691" s="0" t="s">
+        <v>1998</v>
+      </c>
+      <c r="D691" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E691" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F691" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G691" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H691" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I691" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J691" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K691" s="0">
+        <v>27208.47</v>
+      </c>
+      <c r="L691" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M691" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N691" s="0" t="s">
+        <v>1999</v>
+      </c>
+      <c r="O691" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P691" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q691" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R691" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S691" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T691" s="0">
+        <v>3752.9</v>
+      </c>
+      <c r="U691" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V691" s="0">
+        <v>1</v>
+      </c>
+      <c r="W691" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X691" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y691" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z691" s="0">
+        <v>27208.47</v>
+      </c>
+      <c r="AA691" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB691" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC691" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD691" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE691" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF691" s="0" t="s">
+        <v>2000</v>
+      </c>
+      <c r="AG691" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="0">
+        <v>19132</v>
+      </c>
+      <c r="B692" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C692" s="0" t="s">
+        <v>2001</v>
+      </c>
+      <c r="D692" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E692" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F692" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G692" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H692" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I692" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J692" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K692" s="0">
+        <v>21894.44</v>
+      </c>
+      <c r="L692" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M692" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N692" s="0" t="s">
+        <v>2002</v>
+      </c>
+      <c r="O692" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P692" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q692" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R692" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S692" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T692" s="0">
+        <v>3019.93</v>
+      </c>
+      <c r="U692" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V692" s="0">
+        <v>1</v>
+      </c>
+      <c r="W692" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X692" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y692" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z692" s="0">
+        <v>21894.44</v>
+      </c>
+      <c r="AA692" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB692" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC692" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD692" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE692" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF692" s="0" t="s">
+        <v>2003</v>
+      </c>
+      <c r="AG692" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" s="0">
+        <v>19133</v>
+      </c>
+      <c r="B693" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C693" s="0" t="s">
+        <v>2004</v>
+      </c>
+      <c r="D693" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E693" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F693" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G693" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H693" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I693" s="0">
+        <v>20260820</v>
+      </c>
+      <c r="J693" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K693" s="0">
+        <v>96015.89</v>
+      </c>
+      <c r="L693" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M693" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N693" s="0" t="s">
+        <v>2005</v>
+      </c>
+      <c r="O693" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P693" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q693" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R693" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S693" s="0">
+        <v>20260820</v>
+      </c>
+      <c r="T693" s="0">
+        <v>13243.58</v>
+      </c>
+      <c r="U693" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V693" s="0">
+        <v>1</v>
+      </c>
+      <c r="W693" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X693" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y693" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z693" s="0">
+        <v>96015.89</v>
+      </c>
+      <c r="AA693" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB693" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC693" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD693" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE693" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF693" s="0" t="s">
+        <v>2006</v>
+      </c>
+      <c r="AG693" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" s="0">
+        <v>19134</v>
+      </c>
+      <c r="B694" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C694" s="0" t="s">
+        <v>2007</v>
+      </c>
+      <c r="D694" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E694" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F694" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G694" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H694" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I694" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J694" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K694" s="0">
+        <v>123385.23</v>
+      </c>
+      <c r="L694" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M694" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N694" s="0" t="s">
+        <v>2008</v>
+      </c>
+      <c r="O694" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P694" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q694" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R694" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S694" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T694" s="0">
+        <v>17018.66</v>
+      </c>
+      <c r="U694" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V694" s="0">
+        <v>1</v>
+      </c>
+      <c r="W694" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X694" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y694" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z694" s="0">
+        <v>123385.23</v>
+      </c>
+      <c r="AA694" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB694" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC694" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD694" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE694" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF694" s="0" t="s">
+        <v>2009</v>
+      </c>
+      <c r="AG694" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" s="0">
+        <v>19135</v>
+      </c>
+      <c r="B695" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C695" s="0" t="s">
+        <v>2010</v>
+      </c>
+      <c r="D695" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E695" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F695" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G695" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H695" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I695" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J695" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K695" s="0">
+        <v>207850.42</v>
+      </c>
+      <c r="L695" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M695" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N695" s="0" t="s">
+        <v>2011</v>
+      </c>
+      <c r="O695" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P695" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q695" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R695" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S695" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T695" s="0">
+        <v>28669.02</v>
+      </c>
+      <c r="U695" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V695" s="0">
+        <v>1</v>
+      </c>
+      <c r="W695" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X695" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y695" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z695" s="0">
+        <v>207850.42</v>
+      </c>
+      <c r="AA695" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB695" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC695" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD695" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE695" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF695" s="0" t="s">
+        <v>2012</v>
+      </c>
+      <c r="AG695" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" s="0">
+        <v>19136</v>
+      </c>
+      <c r="B696" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C696" s="0" t="s">
+        <v>2013</v>
+      </c>
+      <c r="D696" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E696" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F696" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G696" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H696" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I696" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J696" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K696" s="0">
+        <v>40466.59</v>
+      </c>
+      <c r="L696" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M696" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N696" s="0" t="s">
+        <v>2014</v>
+      </c>
+      <c r="O696" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P696" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q696" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R696" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S696" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T696" s="0">
+        <v>5581.6</v>
+      </c>
+      <c r="U696" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V696" s="0">
+        <v>1</v>
+      </c>
+      <c r="W696" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X696" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y696" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z696" s="0">
+        <v>40466.59</v>
+      </c>
+      <c r="AA696" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB696" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC696" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD696" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE696" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF696" s="0" t="s">
+        <v>2015</v>
+      </c>
+      <c r="AG696" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" s="0">
+        <v>19137</v>
+      </c>
+      <c r="B697" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C697" s="0" t="s">
+        <v>2016</v>
+      </c>
+      <c r="D697" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E697" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F697" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G697" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H697" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I697" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="J697" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K697" s="0">
+        <v>42486.92</v>
+      </c>
+      <c r="L697" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M697" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N697" s="0" t="s">
+        <v>2017</v>
+      </c>
+      <c r="O697" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P697" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q697" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R697" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S697" s="0">
+        <v>20260818</v>
+      </c>
+      <c r="T697" s="0">
+        <v>5860.27</v>
+      </c>
+      <c r="U697" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V697" s="0">
+        <v>1</v>
+      </c>
+      <c r="W697" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X697" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y697" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z697" s="0">
+        <v>42486.92</v>
+      </c>
+      <c r="AA697" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB697" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC697" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD697" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE697" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF697" s="0" t="s">
+        <v>2018</v>
+      </c>
+      <c r="AG697" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" s="0">
+        <v>19138</v>
+      </c>
+      <c r="B698" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C698" s="0" t="s">
+        <v>2019</v>
+      </c>
+      <c r="D698" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E698" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F698" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G698" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H698" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I698" s="0">
+        <v>20260819</v>
+      </c>
+      <c r="J698" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K698" s="0">
+        <v>127934.88</v>
+      </c>
+      <c r="L698" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M698" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N698" s="0" t="s">
+        <v>2020</v>
+      </c>
+      <c r="O698" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P698" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q698" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R698" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S698" s="0">
+        <v>20260819</v>
+      </c>
+      <c r="T698" s="0">
+        <v>17646.19</v>
+      </c>
+      <c r="U698" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V698" s="0">
+        <v>1</v>
+      </c>
+      <c r="W698" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X698" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y698" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z698" s="0">
+        <v>127934.88</v>
+      </c>
+      <c r="AA698" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB698" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC698" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD698" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE698" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF698" s="0" t="s">
+        <v>2021</v>
+      </c>
+      <c r="AG698" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" s="0">
+        <v>19139</v>
+      </c>
+      <c r="B699" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C699" s="0" t="s">
+        <v>2022</v>
+      </c>
+      <c r="D699" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E699" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F699" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G699" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H699" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I699" s="0">
+        <v>20260819</v>
+      </c>
+      <c r="J699" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K699" s="0">
+        <v>78993.2</v>
+      </c>
+      <c r="L699" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M699" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N699" s="0" t="s">
+        <v>2023</v>
+      </c>
+      <c r="O699" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P699" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q699" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R699" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S699" s="0">
+        <v>20260819</v>
+      </c>
+      <c r="T699" s="0">
+        <v>10895.61</v>
+      </c>
+      <c r="U699" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V699" s="0">
+        <v>1</v>
+      </c>
+      <c r="W699" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X699" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y699" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z699" s="0">
+        <v>78993.2</v>
+      </c>
+      <c r="AA699" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB699" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC699" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD699" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE699" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF699" s="0" t="s">
+        <v>2024</v>
+      </c>
+      <c r="AG699" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" s="0">
+        <v>19140</v>
+      </c>
+      <c r="B700" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C700" s="0" t="s">
+        <v>2025</v>
+      </c>
+      <c r="D700" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E700" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F700" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G700" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H700" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I700" s="0">
+        <v>20260820</v>
+      </c>
+      <c r="J700" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K700" s="0">
+        <v>56492.66</v>
+      </c>
+      <c r="L700" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M700" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N700" s="0" t="s">
+        <v>2026</v>
+      </c>
+      <c r="O700" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P700" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q700" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R700" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S700" s="0">
+        <v>20260820</v>
+      </c>
+      <c r="T700" s="0">
+        <v>7792.09</v>
+      </c>
+      <c r="U700" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V700" s="0">
+        <v>1</v>
+      </c>
+      <c r="W700" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X700" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y700" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z700" s="0">
+        <v>56492.66</v>
+      </c>
+      <c r="AA700" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB700" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC700" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD700" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE700" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF700" s="0" t="s">
+        <v>2027</v>
+      </c>
+      <c r="AG700" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" s="0">
+        <v>19141</v>
+      </c>
+      <c r="B701" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C701" s="0" t="s">
+        <v>2028</v>
+      </c>
+      <c r="D701" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E701" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F701" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G701" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H701" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I701" s="0">
+        <v>20260820</v>
+      </c>
+      <c r="J701" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K701" s="0">
+        <v>86393.83</v>
+      </c>
+      <c r="L701" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M701" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N701" s="0" t="s">
+        <v>2029</v>
+      </c>
+      <c r="O701" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P701" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q701" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R701" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S701" s="0">
+        <v>20260820</v>
+      </c>
+      <c r="T701" s="0">
+        <v>11916.39</v>
+      </c>
+      <c r="U701" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V701" s="0">
+        <v>1</v>
+      </c>
+      <c r="W701" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X701" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y701" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z701" s="0">
+        <v>86393.83</v>
+      </c>
+      <c r="AA701" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB701" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC701" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD701" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE701" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF701" s="0" t="s">
+        <v>2030</v>
+      </c>
+      <c r="AG701" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" s="0">
+        <v>19142</v>
+      </c>
+      <c r="B702" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C702" s="0" t="s">
+        <v>2031</v>
+      </c>
+      <c r="D702" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E702" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F702" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G702" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H702" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I702" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="J702" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="K702" s="0">
+        <v>202748.18</v>
+      </c>
+      <c r="L702" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M702" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N702" s="0" t="s">
+        <v>2032</v>
+      </c>
+      <c r="O702" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P702" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q702" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R702" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S702" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="T702" s="0">
+        <v>27965.27</v>
+      </c>
+      <c r="U702" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V702" s="0">
+        <v>1</v>
+      </c>
+      <c r="W702" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X702" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y702" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z702" s="0">
+        <v>202748.18</v>
+      </c>
+      <c r="AA702" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB702" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC702" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD702" s="0">
+        <v>20260821</v>
+      </c>
+      <c r="AE702" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF702" s="0" t="s">
+        <v>2033</v>
+      </c>
+      <c r="AG702" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
   </sheetData>
   <headerFooter/>
 </worksheet>

</xml_diff>

<commit_message>
actualizacion del portal para la subida de informacion
</commit_message>
<xml_diff>
--- a/detecno.xlsx
+++ b/detecno.xlsx
@@ -5,13 +5,13 @@
     <workbookView/>
   </bookViews>
   <sheets>
-    <sheet name="Facturas Seleccionadas" sheetId="1" r:id="R8af8e09dff0a4c8d"/>
+    <sheet name="Facturas Seleccionadas" sheetId="1" r:id="R628ed2d1da074724"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2034" uniqueCount="2034">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2070" uniqueCount="2070">
   <si>
     <t>ID</t>
   </si>
@@ -6113,6 +6113,114 @@
   </si>
   <si>
     <t>4500460559</t>
+  </si>
+  <si>
+    <t>49956</t>
+  </si>
+  <si>
+    <t>65afe28b-cde7-4b31-865e-4ff9980340df</t>
+  </si>
+  <si>
+    <t>E006338824</t>
+  </si>
+  <si>
+    <t>50223</t>
+  </si>
+  <si>
+    <t>951afa1e-9789-4653-ba64-858fde57e300</t>
+  </si>
+  <si>
+    <t>E006342360</t>
+  </si>
+  <si>
+    <t>50224</t>
+  </si>
+  <si>
+    <t>467028fe-6e9f-4f5a-af68-0bbe6e33581a</t>
+  </si>
+  <si>
+    <t>E006342359</t>
+  </si>
+  <si>
+    <t>50285</t>
+  </si>
+  <si>
+    <t>c7dee5b4-2ab3-4f77-81f8-a0c398802c04</t>
+  </si>
+  <si>
+    <t>E006345858</t>
+  </si>
+  <si>
+    <t>50284</t>
+  </si>
+  <si>
+    <t>c00b54d3-10a1-48ee-b398-1e1b9ab8e056</t>
+  </si>
+  <si>
+    <t>E006345859</t>
+  </si>
+  <si>
+    <t>50299</t>
+  </si>
+  <si>
+    <t>1ef7f917-62d3-486f-8353-eb0c70280b3d</t>
+  </si>
+  <si>
+    <t>E006345856</t>
+  </si>
+  <si>
+    <t>50312</t>
+  </si>
+  <si>
+    <t>0ca7c0d9-bf1b-4f2f-9763-6bd07e8137e5</t>
+  </si>
+  <si>
+    <t>4500479274</t>
+  </si>
+  <si>
+    <t>50410</t>
+  </si>
+  <si>
+    <t>2913a99d-adfe-413d-aa82-a61a45ea547a</t>
+  </si>
+  <si>
+    <t>4500472366</t>
+  </si>
+  <si>
+    <t>50198</t>
+  </si>
+  <si>
+    <t>b2070951-5848-4725-8364-3d6a3de4bdf9</t>
+  </si>
+  <si>
+    <t>E006342361</t>
+  </si>
+  <si>
+    <t>50513</t>
+  </si>
+  <si>
+    <t>254b12fe-c46a-47ac-8441-8705cff2f830</t>
+  </si>
+  <si>
+    <t>4500483677</t>
+  </si>
+  <si>
+    <t>50282</t>
+  </si>
+  <si>
+    <t>0c9590be-fdf5-4e17-afad-c2378b24aa71</t>
+  </si>
+  <si>
+    <t>E006345860</t>
+  </si>
+  <si>
+    <t>50296</t>
+  </si>
+  <si>
+    <t>6ad469da-6dd3-4d7f-9890-c3016a9758f0</t>
+  </si>
+  <si>
+    <t>E006345857</t>
   </si>
 </sst>
 </file>
@@ -6158,7 +6266,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AG702"/>
+  <dimension ref="A1:AG714"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.140625" customWidth="1"/>
@@ -77098,6 +77206,1218 @@
         <v>43</v>
       </c>
     </row>
+    <row r="703">
+      <c r="A703" s="0">
+        <v>19375</v>
+      </c>
+      <c r="B703" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C703" s="0" t="s">
+        <v>2034</v>
+      </c>
+      <c r="D703" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E703" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F703" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G703" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H703" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I703" s="0">
+        <v>20260824</v>
+      </c>
+      <c r="J703" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="K703" s="0">
+        <v>13815.7</v>
+      </c>
+      <c r="L703" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M703" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N703" s="0" t="s">
+        <v>2035</v>
+      </c>
+      <c r="O703" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P703" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q703" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R703" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S703" s="0">
+        <v>20260824</v>
+      </c>
+      <c r="T703" s="0">
+        <v>1905.61</v>
+      </c>
+      <c r="U703" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V703" s="0">
+        <v>1</v>
+      </c>
+      <c r="W703" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X703" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y703" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z703" s="0">
+        <v>13815.7</v>
+      </c>
+      <c r="AA703" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB703" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC703" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD703" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="AE703" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF703" s="0" t="s">
+        <v>2036</v>
+      </c>
+      <c r="AG703" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="0">
+        <v>19376</v>
+      </c>
+      <c r="B704" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C704" s="0" t="s">
+        <v>2037</v>
+      </c>
+      <c r="D704" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E704" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F704" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G704" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H704" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I704" s="0">
+        <v>20260826</v>
+      </c>
+      <c r="J704" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="K704" s="0">
+        <v>10365.63</v>
+      </c>
+      <c r="L704" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M704" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N704" s="0" t="s">
+        <v>2038</v>
+      </c>
+      <c r="O704" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P704" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q704" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R704" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S704" s="0">
+        <v>20260826</v>
+      </c>
+      <c r="T704" s="0">
+        <v>1429.74</v>
+      </c>
+      <c r="U704" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V704" s="0">
+        <v>1</v>
+      </c>
+      <c r="W704" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X704" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y704" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z704" s="0">
+        <v>10365.63</v>
+      </c>
+      <c r="AA704" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB704" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC704" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD704" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="AE704" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF704" s="0" t="s">
+        <v>2039</v>
+      </c>
+      <c r="AG704" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="0">
+        <v>19377</v>
+      </c>
+      <c r="B705" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C705" s="0" t="s">
+        <v>2040</v>
+      </c>
+      <c r="D705" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E705" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F705" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G705" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H705" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I705" s="0">
+        <v>20260826</v>
+      </c>
+      <c r="J705" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="K705" s="0">
+        <v>24440.21</v>
+      </c>
+      <c r="L705" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M705" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N705" s="0" t="s">
+        <v>2041</v>
+      </c>
+      <c r="O705" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P705" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q705" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R705" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S705" s="0">
+        <v>20260826</v>
+      </c>
+      <c r="T705" s="0">
+        <v>3371.07</v>
+      </c>
+      <c r="U705" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V705" s="0">
+        <v>1</v>
+      </c>
+      <c r="W705" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X705" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y705" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z705" s="0">
+        <v>24440.21</v>
+      </c>
+      <c r="AA705" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB705" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC705" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD705" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="AE705" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF705" s="0" t="s">
+        <v>2042</v>
+      </c>
+      <c r="AG705" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="0">
+        <v>19378</v>
+      </c>
+      <c r="B706" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C706" s="0" t="s">
+        <v>2043</v>
+      </c>
+      <c r="D706" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E706" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F706" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G706" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H706" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I706" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="J706" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="K706" s="0">
+        <v>18470.75</v>
+      </c>
+      <c r="L706" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M706" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N706" s="0" t="s">
+        <v>2044</v>
+      </c>
+      <c r="O706" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P706" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q706" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R706" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S706" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="T706" s="0">
+        <v>2547.69</v>
+      </c>
+      <c r="U706" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V706" s="0">
+        <v>1</v>
+      </c>
+      <c r="W706" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X706" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y706" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z706" s="0">
+        <v>18470.75</v>
+      </c>
+      <c r="AA706" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB706" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC706" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD706" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="AE706" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF706" s="0" t="s">
+        <v>2045</v>
+      </c>
+      <c r="AG706" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="0">
+        <v>19379</v>
+      </c>
+      <c r="B707" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C707" s="0" t="s">
+        <v>2046</v>
+      </c>
+      <c r="D707" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E707" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F707" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G707" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H707" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I707" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="J707" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="K707" s="0">
+        <v>11541.9</v>
+      </c>
+      <c r="L707" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M707" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N707" s="0" t="s">
+        <v>2047</v>
+      </c>
+      <c r="O707" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P707" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q707" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R707" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S707" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="T707" s="0">
+        <v>1591.99</v>
+      </c>
+      <c r="U707" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V707" s="0">
+        <v>1</v>
+      </c>
+      <c r="W707" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X707" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y707" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z707" s="0">
+        <v>11541.9</v>
+      </c>
+      <c r="AA707" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB707" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC707" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD707" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="AE707" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF707" s="0" t="s">
+        <v>2048</v>
+      </c>
+      <c r="AG707" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" s="0">
+        <v>19380</v>
+      </c>
+      <c r="B708" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C708" s="0" t="s">
+        <v>2049</v>
+      </c>
+      <c r="D708" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E708" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F708" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G708" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H708" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I708" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="J708" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="K708" s="0">
+        <v>6728</v>
+      </c>
+      <c r="L708" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M708" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N708" s="0" t="s">
+        <v>2050</v>
+      </c>
+      <c r="O708" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P708" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q708" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R708" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S708" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="T708" s="0">
+        <v>928</v>
+      </c>
+      <c r="U708" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V708" s="0">
+        <v>1</v>
+      </c>
+      <c r="W708" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X708" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y708" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z708" s="0">
+        <v>6728</v>
+      </c>
+      <c r="AA708" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB708" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC708" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD708" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="AE708" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF708" s="0" t="s">
+        <v>2051</v>
+      </c>
+      <c r="AG708" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" s="0">
+        <v>19381</v>
+      </c>
+      <c r="B709" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C709" s="0" t="s">
+        <v>2052</v>
+      </c>
+      <c r="D709" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E709" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F709" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G709" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H709" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I709" s="0">
+        <v>20260825</v>
+      </c>
+      <c r="J709" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="K709" s="0">
+        <v>83065.2</v>
+      </c>
+      <c r="L709" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M709" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N709" s="0" t="s">
+        <v>2053</v>
+      </c>
+      <c r="O709" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P709" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q709" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R709" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S709" s="0">
+        <v>20260825</v>
+      </c>
+      <c r="T709" s="0">
+        <v>11457.27</v>
+      </c>
+      <c r="U709" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V709" s="0">
+        <v>1</v>
+      </c>
+      <c r="W709" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X709" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y709" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z709" s="0">
+        <v>83065.2</v>
+      </c>
+      <c r="AA709" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB709" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC709" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD709" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="AE709" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF709" s="0" t="s">
+        <v>2054</v>
+      </c>
+      <c r="AG709" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="0">
+        <v>19382</v>
+      </c>
+      <c r="B710" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C710" s="0" t="s">
+        <v>2055</v>
+      </c>
+      <c r="D710" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E710" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F710" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G710" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H710" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I710" s="0">
+        <v>20260826</v>
+      </c>
+      <c r="J710" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="K710" s="0">
+        <v>101082.85</v>
+      </c>
+      <c r="L710" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M710" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N710" s="0" t="s">
+        <v>2056</v>
+      </c>
+      <c r="O710" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P710" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q710" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R710" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S710" s="0">
+        <v>20260826</v>
+      </c>
+      <c r="T710" s="0">
+        <v>13942.46</v>
+      </c>
+      <c r="U710" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V710" s="0">
+        <v>1</v>
+      </c>
+      <c r="W710" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X710" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y710" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z710" s="0">
+        <v>101082.85</v>
+      </c>
+      <c r="AA710" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB710" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC710" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD710" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="AE710" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF710" s="0" t="s">
+        <v>2057</v>
+      </c>
+      <c r="AG710" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="0">
+        <v>19383</v>
+      </c>
+      <c r="B711" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C711" s="0" t="s">
+        <v>2058</v>
+      </c>
+      <c r="D711" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E711" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F711" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G711" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H711" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I711" s="0">
+        <v>20260826</v>
+      </c>
+      <c r="J711" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="K711" s="0">
+        <v>14644.25</v>
+      </c>
+      <c r="L711" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M711" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N711" s="0" t="s">
+        <v>2059</v>
+      </c>
+      <c r="O711" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P711" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q711" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R711" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S711" s="0">
+        <v>20260826</v>
+      </c>
+      <c r="T711" s="0">
+        <v>2019.9</v>
+      </c>
+      <c r="U711" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V711" s="0">
+        <v>1</v>
+      </c>
+      <c r="W711" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X711" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y711" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z711" s="0">
+        <v>14644.25</v>
+      </c>
+      <c r="AA711" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB711" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC711" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD711" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="AE711" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF711" s="0" t="s">
+        <v>2060</v>
+      </c>
+      <c r="AG711" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="0">
+        <v>19384</v>
+      </c>
+      <c r="B712" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C712" s="0" t="s">
+        <v>2061</v>
+      </c>
+      <c r="D712" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E712" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F712" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G712" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H712" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I712" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="J712" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="K712" s="0">
+        <v>7145.6</v>
+      </c>
+      <c r="L712" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M712" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N712" s="0" t="s">
+        <v>2062</v>
+      </c>
+      <c r="O712" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P712" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q712" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R712" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S712" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="T712" s="0">
+        <v>985.6</v>
+      </c>
+      <c r="U712" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V712" s="0">
+        <v>1</v>
+      </c>
+      <c r="W712" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X712" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y712" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z712" s="0">
+        <v>7145.6</v>
+      </c>
+      <c r="AA712" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB712" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC712" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD712" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="AE712" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF712" s="0" t="s">
+        <v>2063</v>
+      </c>
+      <c r="AG712" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="0">
+        <v>19385</v>
+      </c>
+      <c r="B713" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C713" s="0" t="s">
+        <v>2064</v>
+      </c>
+      <c r="D713" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E713" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F713" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G713" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H713" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I713" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="J713" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="K713" s="0">
+        <v>17685.4</v>
+      </c>
+      <c r="L713" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M713" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N713" s="0" t="s">
+        <v>2065</v>
+      </c>
+      <c r="O713" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P713" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q713" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R713" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S713" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="T713" s="0">
+        <v>2439.37</v>
+      </c>
+      <c r="U713" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V713" s="0">
+        <v>1</v>
+      </c>
+      <c r="W713" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X713" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y713" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z713" s="0">
+        <v>17685.4</v>
+      </c>
+      <c r="AA713" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB713" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC713" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD713" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="AE713" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF713" s="0" t="s">
+        <v>2066</v>
+      </c>
+      <c r="AG713" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="0">
+        <v>19386</v>
+      </c>
+      <c r="B714" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C714" s="0" t="s">
+        <v>2067</v>
+      </c>
+      <c r="D714" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E714" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F714" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G714" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H714" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I714" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="J714" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="K714" s="0">
+        <v>6728</v>
+      </c>
+      <c r="L714" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M714" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N714" s="0" t="s">
+        <v>2068</v>
+      </c>
+      <c r="O714" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P714" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q714" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R714" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S714" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="T714" s="0">
+        <v>928</v>
+      </c>
+      <c r="U714" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V714" s="0">
+        <v>1</v>
+      </c>
+      <c r="W714" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X714" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y714" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z714" s="0">
+        <v>6728</v>
+      </c>
+      <c r="AA714" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB714" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC714" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD714" s="0">
+        <v>20260828</v>
+      </c>
+      <c r="AE714" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF714" s="0" t="s">
+        <v>2069</v>
+      </c>
+      <c r="AG714" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
   </sheetData>
   <headerFooter/>
 </worksheet>

</xml_diff>

<commit_message>
reporte de la semana con modificaciones a la sua de base de datos
</commit_message>
<xml_diff>
--- a/detecno.xlsx
+++ b/detecno.xlsx
@@ -5,13 +5,13 @@
     <workbookView/>
   </bookViews>
   <sheets>
-    <sheet name="Facturas Seleccionadas" sheetId="1" r:id="R628ed2d1da074724"/>
+    <sheet name="Facturas Seleccionadas" sheetId="1" r:id="R77ac216a50d246c2"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2070" uniqueCount="2070">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2121" uniqueCount="2121">
   <si>
     <t>ID</t>
   </si>
@@ -6221,6 +6221,159 @@
   </si>
   <si>
     <t>E006345857</t>
+  </si>
+  <si>
+    <t>50298</t>
+  </si>
+  <si>
+    <t>4c956a33-513f-4bd0-b67e-95da954364fe</t>
+  </si>
+  <si>
+    <t>E006348983</t>
+  </si>
+  <si>
+    <t>50415</t>
+  </si>
+  <si>
+    <t>b01fd6a2-9ff6-4d5a-a4ae-88a1ef023575</t>
+  </si>
+  <si>
+    <t>E006348985</t>
+  </si>
+  <si>
+    <t>50512</t>
+  </si>
+  <si>
+    <t>a26efb0b-637f-4c84-bad7-3fbe1d20d979</t>
+  </si>
+  <si>
+    <t>E006348987</t>
+  </si>
+  <si>
+    <t>50572</t>
+  </si>
+  <si>
+    <t>7b9727fd-d5da-4ce4-901c-f397b003678a</t>
+  </si>
+  <si>
+    <t>E006350642</t>
+  </si>
+  <si>
+    <t>50636</t>
+  </si>
+  <si>
+    <t>c0ba297f-bbfb-4f70-8a80-f968957bf7a8</t>
+  </si>
+  <si>
+    <t>E006352349</t>
+  </si>
+  <si>
+    <t>50637</t>
+  </si>
+  <si>
+    <t>56595d64-c9a5-4abf-8751-20aa983988e0</t>
+  </si>
+  <si>
+    <t>E006352358</t>
+  </si>
+  <si>
+    <t>50631</t>
+  </si>
+  <si>
+    <t>006e10e1-570e-4471-8342-d0a417bca093</t>
+  </si>
+  <si>
+    <t>4500460814</t>
+  </si>
+  <si>
+    <t>50633</t>
+  </si>
+  <si>
+    <t>c5b06034-7454-45e0-b1c3-729bbb5b804d</t>
+  </si>
+  <si>
+    <t>4500464707</t>
+  </si>
+  <si>
+    <t>50095</t>
+  </si>
+  <si>
+    <t>6cf8b06c-79c9-4ddd-8b22-d50ff9915b06</t>
+  </si>
+  <si>
+    <t>E006348990</t>
+  </si>
+  <si>
+    <t>50413</t>
+  </si>
+  <si>
+    <t>aa327423-2675-4896-b2d2-aae586435b18</t>
+  </si>
+  <si>
+    <t>E006348986</t>
+  </si>
+  <si>
+    <t>50564</t>
+  </si>
+  <si>
+    <t>246e56be-e91a-441b-abf1-28ccd06e20e1</t>
+  </si>
+  <si>
+    <t>E006350644</t>
+  </si>
+  <si>
+    <t>50472</t>
+  </si>
+  <si>
+    <t>3dfa5719-1985-42e7-b580-7744f2bada14</t>
+  </si>
+  <si>
+    <t>E006348988</t>
+  </si>
+  <si>
+    <t>50749</t>
+  </si>
+  <si>
+    <t>a4f4bde7-4c2b-49ab-8538-04c530804d4d</t>
+  </si>
+  <si>
+    <t>4500462199</t>
+  </si>
+  <si>
+    <t>50750</t>
+  </si>
+  <si>
+    <t>080e9e65-1a39-452b-9011-79088ec7d793</t>
+  </si>
+  <si>
+    <t>4500483424</t>
+  </si>
+  <si>
+    <t>50700</t>
+  </si>
+  <si>
+    <t>639c619c-0186-41c8-bc96-609c3ce38181</t>
+  </si>
+  <si>
+    <t>4500485292</t>
+  </si>
+  <si>
+    <t>50707</t>
+  </si>
+  <si>
+    <t>d8ffb7a1-1c06-4688-9cf6-0b8fd7b37873</t>
+  </si>
+  <si>
+    <t>4500487967</t>
+  </si>
+  <si>
+    <t>50676</t>
+  </si>
+  <si>
+    <t>0053d8c4-5252-4e85-9b3b-3eeeee5dc8fc</t>
+  </si>
+  <si>
+    <t>E006354202</t>
   </si>
 </sst>
 </file>
@@ -6266,7 +6419,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AG714"/>
+  <dimension ref="A1:AG731"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.140625" customWidth="1"/>
@@ -78418,6 +78571,1723 @@
         <v>43</v>
       </c>
     </row>
+    <row r="715">
+      <c r="A715" s="0">
+        <v>19572</v>
+      </c>
+      <c r="B715" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C715" s="0" t="s">
+        <v>2070</v>
+      </c>
+      <c r="D715" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E715" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F715" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G715" s="0" t="s">
+        <v>560</v>
+      </c>
+      <c r="H715" s="0" t="s">
+        <v>561</v>
+      </c>
+      <c r="I715" s="0">
+        <v>20260901</v>
+      </c>
+      <c r="J715" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="K715" s="0">
+        <v>6728</v>
+      </c>
+      <c r="L715" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M715" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N715" s="0" t="s">
+        <v>2071</v>
+      </c>
+      <c r="O715" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P715" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q715" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R715" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S715" s="0">
+        <v>20260901</v>
+      </c>
+      <c r="T715" s="0">
+        <v>928</v>
+      </c>
+      <c r="U715" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V715" s="0">
+        <v>1</v>
+      </c>
+      <c r="W715" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X715" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y715" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z715" s="0">
+        <v>6728</v>
+      </c>
+      <c r="AA715" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB715" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC715" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD715" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="AE715" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF715" s="0" t="s">
+        <v>2072</v>
+      </c>
+      <c r="AG715" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="0">
+        <v>19573</v>
+      </c>
+      <c r="B716" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C716" s="0" t="s">
+        <v>2073</v>
+      </c>
+      <c r="D716" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E716" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F716" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G716" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H716" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I716" s="0">
+        <v>20260901</v>
+      </c>
+      <c r="J716" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="K716" s="0">
+        <v>20008.92</v>
+      </c>
+      <c r="L716" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M716" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N716" s="0" t="s">
+        <v>2074</v>
+      </c>
+      <c r="O716" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P716" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q716" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R716" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S716" s="0">
+        <v>20260901</v>
+      </c>
+      <c r="T716" s="0">
+        <v>2759.85</v>
+      </c>
+      <c r="U716" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V716" s="0">
+        <v>1</v>
+      </c>
+      <c r="W716" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X716" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y716" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z716" s="0">
+        <v>20008.92</v>
+      </c>
+      <c r="AA716" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB716" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC716" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD716" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="AE716" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF716" s="0" t="s">
+        <v>2075</v>
+      </c>
+      <c r="AG716" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="0">
+        <v>19574</v>
+      </c>
+      <c r="B717" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C717" s="0" t="s">
+        <v>2076</v>
+      </c>
+      <c r="D717" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E717" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F717" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G717" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H717" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I717" s="0">
+        <v>20260901</v>
+      </c>
+      <c r="J717" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="K717" s="0">
+        <v>21884.38</v>
+      </c>
+      <c r="L717" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M717" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N717" s="0" t="s">
+        <v>2077</v>
+      </c>
+      <c r="O717" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P717" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q717" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R717" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S717" s="0">
+        <v>20260901</v>
+      </c>
+      <c r="T717" s="0">
+        <v>3018.54</v>
+      </c>
+      <c r="U717" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V717" s="0">
+        <v>1</v>
+      </c>
+      <c r="W717" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X717" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y717" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z717" s="0">
+        <v>21884.38</v>
+      </c>
+      <c r="AA717" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB717" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC717" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD717" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="AE717" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF717" s="0" t="s">
+        <v>2078</v>
+      </c>
+      <c r="AG717" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="0">
+        <v>19575</v>
+      </c>
+      <c r="B718" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C718" s="0" t="s">
+        <v>2079</v>
+      </c>
+      <c r="D718" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E718" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F718" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G718" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H718" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I718" s="0">
+        <v>20260902</v>
+      </c>
+      <c r="J718" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="K718" s="0">
+        <v>15967.12</v>
+      </c>
+      <c r="L718" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M718" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N718" s="0" t="s">
+        <v>2080</v>
+      </c>
+      <c r="O718" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P718" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q718" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R718" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S718" s="0">
+        <v>20260902</v>
+      </c>
+      <c r="T718" s="0">
+        <v>2202.37</v>
+      </c>
+      <c r="U718" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V718" s="0">
+        <v>1</v>
+      </c>
+      <c r="W718" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X718" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y718" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z718" s="0">
+        <v>15967.12</v>
+      </c>
+      <c r="AA718" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB718" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC718" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD718" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="AE718" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF718" s="0" t="s">
+        <v>2081</v>
+      </c>
+      <c r="AG718" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" s="0">
+        <v>19576</v>
+      </c>
+      <c r="B719" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C719" s="0" t="s">
+        <v>2082</v>
+      </c>
+      <c r="D719" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E719" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F719" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G719" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H719" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I719" s="0">
+        <v>20260903</v>
+      </c>
+      <c r="J719" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="K719" s="0">
+        <v>17685.4</v>
+      </c>
+      <c r="L719" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M719" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N719" s="0" t="s">
+        <v>2083</v>
+      </c>
+      <c r="O719" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P719" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q719" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R719" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S719" s="0">
+        <v>20260903</v>
+      </c>
+      <c r="T719" s="0">
+        <v>2439.37</v>
+      </c>
+      <c r="U719" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V719" s="0">
+        <v>1</v>
+      </c>
+      <c r="W719" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X719" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y719" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z719" s="0">
+        <v>17685.4</v>
+      </c>
+      <c r="AA719" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB719" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC719" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD719" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="AE719" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF719" s="0" t="s">
+        <v>2084</v>
+      </c>
+      <c r="AG719" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" s="0">
+        <v>19577</v>
+      </c>
+      <c r="B720" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C720" s="0" t="s">
+        <v>2085</v>
+      </c>
+      <c r="D720" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E720" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F720" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G720" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H720" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I720" s="0">
+        <v>20260903</v>
+      </c>
+      <c r="J720" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="K720" s="0">
+        <v>17685.4</v>
+      </c>
+      <c r="L720" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M720" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N720" s="0" t="s">
+        <v>2086</v>
+      </c>
+      <c r="O720" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P720" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q720" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R720" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S720" s="0">
+        <v>20260903</v>
+      </c>
+      <c r="T720" s="0">
+        <v>2439.37</v>
+      </c>
+      <c r="U720" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V720" s="0">
+        <v>1</v>
+      </c>
+      <c r="W720" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X720" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y720" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z720" s="0">
+        <v>17685.4</v>
+      </c>
+      <c r="AA720" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB720" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC720" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD720" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="AE720" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF720" s="0" t="s">
+        <v>2087</v>
+      </c>
+      <c r="AG720" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="0">
+        <v>19578</v>
+      </c>
+      <c r="B721" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C721" s="0" t="s">
+        <v>2088</v>
+      </c>
+      <c r="D721" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E721" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F721" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G721" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H721" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I721" s="0">
+        <v>20260901</v>
+      </c>
+      <c r="J721" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="K721" s="0">
+        <v>137904.91</v>
+      </c>
+      <c r="L721" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M721" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N721" s="0" t="s">
+        <v>2089</v>
+      </c>
+      <c r="O721" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P721" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q721" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R721" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S721" s="0">
+        <v>20260901</v>
+      </c>
+      <c r="T721" s="0">
+        <v>19021.37</v>
+      </c>
+      <c r="U721" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V721" s="0">
+        <v>1</v>
+      </c>
+      <c r="W721" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X721" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y721" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z721" s="0">
+        <v>137904.91</v>
+      </c>
+      <c r="AA721" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB721" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC721" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD721" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="AE721" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF721" s="0" t="s">
+        <v>2090</v>
+      </c>
+      <c r="AG721" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="0">
+        <v>19579</v>
+      </c>
+      <c r="B722" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C722" s="0" t="s">
+        <v>2091</v>
+      </c>
+      <c r="D722" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E722" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F722" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G722" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H722" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I722" s="0">
+        <v>20260901</v>
+      </c>
+      <c r="J722" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="K722" s="0">
+        <v>128430.03</v>
+      </c>
+      <c r="L722" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M722" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N722" s="0" t="s">
+        <v>2092</v>
+      </c>
+      <c r="O722" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P722" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q722" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R722" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S722" s="0">
+        <v>20260901</v>
+      </c>
+      <c r="T722" s="0">
+        <v>17714.49</v>
+      </c>
+      <c r="U722" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V722" s="0">
+        <v>1</v>
+      </c>
+      <c r="W722" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X722" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y722" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z722" s="0">
+        <v>128430.03</v>
+      </c>
+      <c r="AA722" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB722" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC722" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD722" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="AE722" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF722" s="0" t="s">
+        <v>2093</v>
+      </c>
+      <c r="AG722" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" s="0">
+        <v>19580</v>
+      </c>
+      <c r="B723" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C723" s="0" t="s">
+        <v>2094</v>
+      </c>
+      <c r="D723" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E723" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F723" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G723" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H723" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I723" s="0">
+        <v>20260901</v>
+      </c>
+      <c r="J723" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="K723" s="0">
+        <v>4881.23</v>
+      </c>
+      <c r="L723" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M723" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N723" s="0" t="s">
+        <v>2095</v>
+      </c>
+      <c r="O723" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P723" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q723" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R723" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S723" s="0">
+        <v>20260901</v>
+      </c>
+      <c r="T723" s="0">
+        <v>673.27</v>
+      </c>
+      <c r="U723" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V723" s="0">
+        <v>1</v>
+      </c>
+      <c r="W723" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X723" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y723" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z723" s="0">
+        <v>4881.23</v>
+      </c>
+      <c r="AA723" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB723" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC723" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD723" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="AE723" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF723" s="0" t="s">
+        <v>2096</v>
+      </c>
+      <c r="AG723" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" s="0">
+        <v>19581</v>
+      </c>
+      <c r="B724" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C724" s="0" t="s">
+        <v>2097</v>
+      </c>
+      <c r="D724" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E724" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F724" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G724" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H724" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I724" s="0">
+        <v>20260901</v>
+      </c>
+      <c r="J724" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="K724" s="0">
+        <v>19460.46</v>
+      </c>
+      <c r="L724" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M724" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N724" s="0" t="s">
+        <v>2098</v>
+      </c>
+      <c r="O724" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P724" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q724" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R724" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S724" s="0">
+        <v>20260901</v>
+      </c>
+      <c r="T724" s="0">
+        <v>2684.2</v>
+      </c>
+      <c r="U724" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V724" s="0">
+        <v>1</v>
+      </c>
+      <c r="W724" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X724" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y724" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z724" s="0">
+        <v>19460.46</v>
+      </c>
+      <c r="AA724" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB724" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC724" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD724" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="AE724" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF724" s="0" t="s">
+        <v>2099</v>
+      </c>
+      <c r="AG724" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="0">
+        <v>19582</v>
+      </c>
+      <c r="B725" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C725" s="0" t="s">
+        <v>2100</v>
+      </c>
+      <c r="D725" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E725" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F725" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G725" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H725" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I725" s="0">
+        <v>20260902</v>
+      </c>
+      <c r="J725" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="K725" s="0">
+        <v>27242.18</v>
+      </c>
+      <c r="L725" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M725" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N725" s="0" t="s">
+        <v>2101</v>
+      </c>
+      <c r="O725" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P725" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q725" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R725" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S725" s="0">
+        <v>20260902</v>
+      </c>
+      <c r="T725" s="0">
+        <v>3757.54</v>
+      </c>
+      <c r="U725" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V725" s="0">
+        <v>1</v>
+      </c>
+      <c r="W725" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X725" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y725" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z725" s="0">
+        <v>27242.18</v>
+      </c>
+      <c r="AA725" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB725" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC725" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD725" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="AE725" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF725" s="0" t="s">
+        <v>2102</v>
+      </c>
+      <c r="AG725" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="0">
+        <v>19583</v>
+      </c>
+      <c r="B726" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C726" s="0" t="s">
+        <v>2103</v>
+      </c>
+      <c r="D726" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E726" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F726" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G726" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H726" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I726" s="0">
+        <v>20260901</v>
+      </c>
+      <c r="J726" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="K726" s="0">
+        <v>7305.63</v>
+      </c>
+      <c r="L726" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M726" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N726" s="0" t="s">
+        <v>2104</v>
+      </c>
+      <c r="O726" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P726" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q726" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R726" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S726" s="0">
+        <v>20260901</v>
+      </c>
+      <c r="T726" s="0">
+        <v>1007.67</v>
+      </c>
+      <c r="U726" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V726" s="0">
+        <v>1</v>
+      </c>
+      <c r="W726" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X726" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y726" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z726" s="0">
+        <v>7305.63</v>
+      </c>
+      <c r="AA726" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB726" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC726" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD726" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="AE726" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF726" s="0" t="s">
+        <v>2105</v>
+      </c>
+      <c r="AG726" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" s="0">
+        <v>19584</v>
+      </c>
+      <c r="B727" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C727" s="0" t="s">
+        <v>2106</v>
+      </c>
+      <c r="D727" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E727" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F727" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G727" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H727" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I727" s="0">
+        <v>20260903</v>
+      </c>
+      <c r="J727" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="K727" s="0">
+        <v>129508.51</v>
+      </c>
+      <c r="L727" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M727" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N727" s="0" t="s">
+        <v>2107</v>
+      </c>
+      <c r="O727" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P727" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q727" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R727" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S727" s="0">
+        <v>20260903</v>
+      </c>
+      <c r="T727" s="0">
+        <v>17863.24</v>
+      </c>
+      <c r="U727" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V727" s="0">
+        <v>1</v>
+      </c>
+      <c r="W727" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X727" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y727" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z727" s="0">
+        <v>129508.51</v>
+      </c>
+      <c r="AA727" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB727" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC727" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD727" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="AE727" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF727" s="0" t="s">
+        <v>2108</v>
+      </c>
+      <c r="AG727" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" s="0">
+        <v>19585</v>
+      </c>
+      <c r="B728" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C728" s="0" t="s">
+        <v>2109</v>
+      </c>
+      <c r="D728" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E728" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F728" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G728" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H728" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I728" s="0">
+        <v>20260903</v>
+      </c>
+      <c r="J728" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="K728" s="0">
+        <v>49014.8</v>
+      </c>
+      <c r="L728" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M728" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N728" s="0" t="s">
+        <v>2110</v>
+      </c>
+      <c r="O728" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P728" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q728" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R728" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S728" s="0">
+        <v>20260903</v>
+      </c>
+      <c r="T728" s="0">
+        <v>6760.66</v>
+      </c>
+      <c r="U728" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V728" s="0">
+        <v>1</v>
+      </c>
+      <c r="W728" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X728" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y728" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z728" s="0">
+        <v>49014.8</v>
+      </c>
+      <c r="AA728" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB728" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC728" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD728" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="AE728" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF728" s="0" t="s">
+        <v>2111</v>
+      </c>
+      <c r="AG728" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="0">
+        <v>19586</v>
+      </c>
+      <c r="B729" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C729" s="0" t="s">
+        <v>2112</v>
+      </c>
+      <c r="D729" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E729" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F729" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G729" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H729" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I729" s="0">
+        <v>20260903</v>
+      </c>
+      <c r="J729" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="K729" s="0">
+        <v>46543.2</v>
+      </c>
+      <c r="L729" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M729" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N729" s="0" t="s">
+        <v>2113</v>
+      </c>
+      <c r="O729" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P729" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q729" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R729" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S729" s="0">
+        <v>20260903</v>
+      </c>
+      <c r="T729" s="0">
+        <v>6419.75</v>
+      </c>
+      <c r="U729" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V729" s="0">
+        <v>1</v>
+      </c>
+      <c r="W729" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X729" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y729" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z729" s="0">
+        <v>46543.2</v>
+      </c>
+      <c r="AA729" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB729" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC729" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD729" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="AE729" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF729" s="0" t="s">
+        <v>2114</v>
+      </c>
+      <c r="AG729" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" s="0">
+        <v>19587</v>
+      </c>
+      <c r="B730" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C730" s="0" t="s">
+        <v>2115</v>
+      </c>
+      <c r="D730" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E730" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F730" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G730" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H730" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I730" s="0">
+        <v>20260903</v>
+      </c>
+      <c r="J730" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="K730" s="0">
+        <v>28284.47</v>
+      </c>
+      <c r="L730" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M730" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N730" s="0" t="s">
+        <v>2116</v>
+      </c>
+      <c r="O730" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P730" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q730" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R730" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S730" s="0">
+        <v>20260903</v>
+      </c>
+      <c r="T730" s="0">
+        <v>3901.31</v>
+      </c>
+      <c r="U730" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V730" s="0">
+        <v>1</v>
+      </c>
+      <c r="W730" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X730" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y730" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z730" s="0">
+        <v>28284.47</v>
+      </c>
+      <c r="AA730" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB730" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC730" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD730" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="AE730" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF730" s="0" t="s">
+        <v>2117</v>
+      </c>
+      <c r="AG730" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" s="0">
+        <v>19588</v>
+      </c>
+      <c r="B731" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C731" s="0" t="s">
+        <v>2118</v>
+      </c>
+      <c r="D731" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="E731" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F731" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G731" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H731" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I731" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="J731" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="K731" s="0">
+        <v>19424.5</v>
+      </c>
+      <c r="L731" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="M731" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="N731" s="0" t="s">
+        <v>2119</v>
+      </c>
+      <c r="O731" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="P731" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q731" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="R731" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="S731" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="T731" s="0">
+        <v>2679.24</v>
+      </c>
+      <c r="U731" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V731" s="0">
+        <v>1</v>
+      </c>
+      <c r="W731" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="X731" s="0">
+        <v>0</v>
+      </c>
+      <c r="Y731" s="0">
+        <v>0</v>
+      </c>
+      <c r="Z731" s="0">
+        <v>19424.5</v>
+      </c>
+      <c r="AA731" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB731" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC731" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD731" s="0">
+        <v>20260904</v>
+      </c>
+      <c r="AE731" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF731" s="0" t="s">
+        <v>2120</v>
+      </c>
+      <c r="AG731" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
   </sheetData>
   <headerFooter/>
 </worksheet>

</xml_diff>